<commit_message>
Made latest changes in the script till 28 Jan
</commit_message>
<xml_diff>
--- a/data/processed/itasset_col.xlsx
+++ b/data/processed/itasset_col.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\S7NM\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\S7NM\Desktop\EOSL\data\processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A1DA26B-E72F-43F8-AC62-6BBBC5F45226}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8142E0FB-DDEE-4D70-A182-4EB273F6E7DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{22BD5A8C-4A1E-41AD-BCC6-53263153DC52}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{22BD5A8C-4A1E-41AD-BCC6-53263153DC52}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="Sheet4" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -712,7 +713,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -760,12 +761,6 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -846,7 +841,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -899,7 +894,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1250,15 +1244,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E61374A-1B79-4A92-A045-E4BBD1C39B6E}">
   <dimension ref="A1:E114"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="40.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="40.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.44140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1266,7 +1260,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -1274,7 +1268,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1282,7 +1276,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
@@ -1290,7 +1284,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
@@ -1298,7 +1292,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>9</v>
       </c>
@@ -1309,7 +1303,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
@@ -1317,7 +1311,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
@@ -1325,7 +1319,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>16</v>
       </c>
@@ -1333,7 +1327,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>18</v>
       </c>
@@ -1341,7 +1335,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
@@ -1349,7 +1343,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>22</v>
       </c>
@@ -1357,7 +1351,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>24</v>
       </c>
@@ -1365,7 +1359,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>26</v>
       </c>
@@ -1373,7 +1367,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>28</v>
       </c>
@@ -1381,7 +1375,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>30</v>
       </c>
@@ -1389,7 +1383,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
         <v>32</v>
       </c>
@@ -1400,7 +1394,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>35</v>
       </c>
@@ -1408,7 +1402,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>37</v>
       </c>
@@ -1416,7 +1410,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>39</v>
       </c>
@@ -1424,7 +1418,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>41</v>
       </c>
@@ -1432,7 +1426,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>43</v>
       </c>
@@ -1440,7 +1434,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>45</v>
       </c>
@@ -1448,7 +1442,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
         <v>47</v>
       </c>
@@ -1456,7 +1450,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
         <v>49</v>
       </c>
@@ -1467,7 +1461,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>52</v>
       </c>
@@ -1475,7 +1469,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>54</v>
       </c>
@@ -1483,7 +1477,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>55</v>
       </c>
@@ -1491,7 +1485,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>56</v>
       </c>
@@ -1499,7 +1493,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>58</v>
       </c>
@@ -1507,7 +1501,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
         <v>60</v>
       </c>
@@ -1515,7 +1509,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>62</v>
       </c>
@@ -1523,7 +1517,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>64</v>
       </c>
@@ -1531,7 +1525,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" s="5" t="s">
         <v>66</v>
       </c>
@@ -1542,7 +1536,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>69</v>
       </c>
@@ -1550,7 +1544,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
         <v>71</v>
       </c>
@@ -1558,7 +1552,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
         <v>73</v>
       </c>
@@ -1566,7 +1560,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
         <v>75</v>
       </c>
@@ -1577,7 +1571,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
         <v>77</v>
       </c>
@@ -1585,7 +1579,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
         <v>79</v>
       </c>
@@ -1593,7 +1587,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" s="5" t="s">
         <v>81</v>
       </c>
@@ -1604,7 +1598,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
         <v>83</v>
       </c>
@@ -1612,7 +1606,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
         <v>85</v>
       </c>
@@ -1620,7 +1614,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
         <v>87</v>
       </c>
@@ -1628,7 +1622,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
         <v>89</v>
       </c>
@@ -1636,7 +1630,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
         <v>91</v>
       </c>
@@ -1647,7 +1641,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
         <v>94</v>
       </c>
@@ -1655,7 +1649,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48" s="5" t="s">
         <v>95</v>
       </c>
@@ -1666,7 +1660,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" s="5" t="s">
         <v>96</v>
       </c>
@@ -1677,7 +1671,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" s="5" t="s">
         <v>98</v>
       </c>
@@ -1688,7 +1682,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51" s="5" t="s">
         <v>100</v>
       </c>
@@ -1699,7 +1693,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" s="5" t="s">
         <v>102</v>
       </c>
@@ -1710,7 +1704,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53" s="5" t="s">
         <v>104</v>
       </c>
@@ -1721,7 +1715,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" s="5" t="s">
         <v>106</v>
       </c>
@@ -1735,7 +1729,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
         <v>108</v>
       </c>
@@ -1743,7 +1737,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" s="5" t="s">
         <v>110</v>
       </c>
@@ -1754,7 +1748,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
         <v>112</v>
       </c>
@@ -1762,7 +1756,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58" s="5" t="s">
         <v>114</v>
       </c>
@@ -1773,7 +1767,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
         <v>116</v>
       </c>
@@ -1781,7 +1775,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
         <v>118</v>
       </c>
@@ -1789,7 +1783,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
         <v>120</v>
       </c>
@@ -1797,57 +1791,57 @@
         <v>121</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63" s="1" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A65" s="1" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A66" s="1" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A67" s="1" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A68" s="1" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A69" s="1" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A70" s="1" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A71" s="1" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A72" s="5" t="s">
         <v>132</v>
       </c>
@@ -1855,17 +1849,17 @@
         <v>50</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A73" s="1" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A74" s="1" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A75" s="5" t="s">
         <v>135</v>
       </c>
@@ -1873,17 +1867,17 @@
         <v>53</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A76" s="1" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A77" s="1" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A78" s="5" t="s">
         <v>138</v>
       </c>
@@ -1891,32 +1885,32 @@
         <v>82</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A79" s="1" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A80" s="1" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A81" s="1" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A82" s="1" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A83" s="1" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A84" s="5" t="s">
         <v>144</v>
       </c>
@@ -1924,12 +1918,12 @@
         <v>67</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A85" s="1" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A86" s="5" t="s">
         <v>146</v>
       </c>
@@ -1937,27 +1931,27 @@
         <v>105</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A87" s="1" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A88" s="1" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A89" s="1" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A90" s="1" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A91" s="5" t="s">
         <v>151</v>
       </c>
@@ -1965,12 +1959,12 @@
         <v>113</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A92" s="1" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A93" s="5" t="s">
         <v>153</v>
       </c>
@@ -1978,7 +1972,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A94" s="5" t="s">
         <v>154</v>
       </c>
@@ -1986,7 +1980,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A95" s="5" t="s">
         <v>155</v>
       </c>
@@ -1994,12 +1988,12 @@
         <v>107</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A96" s="1" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A97" s="5" t="s">
         <v>157</v>
       </c>
@@ -2007,12 +2001,12 @@
         <v>111</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A98" s="1" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A99" s="5" t="s">
         <v>159</v>
       </c>
@@ -2020,77 +2014,77 @@
         <v>57</v>
       </c>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A100" s="1" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A101" s="1" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A102" s="1" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A103" s="1" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A104" s="1" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A105" s="1" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A106" s="1" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A107" s="1" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A108" s="1" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A109" s="1" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A110" s="1" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A111" s="1" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A112" s="1" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A113" s="1" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="114" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A114" s="1" t="s">
         <v>174</v>
       </c>
@@ -2106,7 +2100,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2DB512E-F7CA-443A-B821-976DCEDFC456}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2115,17 +2109,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D1D4B5F-B204-4612-9FFD-1BD2DC74471D}">
   <dimension ref="A1:H28"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="28.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="33.7109375" customWidth="1"/>
-    <col min="5" max="5" width="30.140625" customWidth="1"/>
-    <col min="7" max="7" width="28.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33.6640625" customWidth="1"/>
+    <col min="5" max="5" width="30.109375" customWidth="1"/>
+    <col min="7" max="7" width="28.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>144</v>
       </c>
@@ -2145,7 +2139,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>159</v>
       </c>
@@ -2165,7 +2159,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>118</v>
       </c>
@@ -2185,7 +2179,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>98</v>
       </c>
@@ -2205,7 +2199,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>146</v>
       </c>
@@ -2225,7 +2219,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>32</v>
       </c>
@@ -2245,7 +2239,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>47</v>
       </c>
@@ -2265,7 +2259,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>66</v>
       </c>
@@ -2285,7 +2279,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>151</v>
       </c>
@@ -2305,7 +2299,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>153</v>
       </c>
@@ -2325,7 +2319,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>155</v>
       </c>
@@ -2345,7 +2339,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>154</v>
       </c>
@@ -2365,7 +2359,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>157</v>
       </c>
@@ -2385,7 +2379,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>106</v>
       </c>
@@ -2405,7 +2399,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
         <v>96</v>
       </c>
@@ -2425,7 +2419,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
         <v>100</v>
       </c>
@@ -2445,7 +2439,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
         <v>102</v>
       </c>
@@ -2465,7 +2459,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
         <v>104</v>
       </c>
@@ -2485,7 +2479,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
         <v>106</v>
       </c>
@@ -2505,7 +2499,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
         <v>110</v>
       </c>
@@ -2525,7 +2519,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
         <v>49</v>
       </c>
@@ -2545,7 +2539,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
         <v>114</v>
       </c>
@@ -2565,7 +2559,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
         <v>81</v>
       </c>
@@ -2585,7 +2579,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
         <v>95</v>
       </c>
@@ -2605,7 +2599,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
         <v>132</v>
       </c>
@@ -2625,7 +2619,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
         <v>9</v>
       </c>
@@ -2645,7 +2639,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
         <v>135</v>
       </c>
@@ -2665,7 +2659,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
         <v>138</v>
       </c>
@@ -2696,34 +2690,34 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF4835EC-2A0F-402C-85DF-9EA38234F424}">
   <dimension ref="A1:G61"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="31.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="32.140625" customWidth="1"/>
-    <col min="3" max="3" width="25.28515625" customWidth="1"/>
+    <col min="1" max="1" width="31.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.109375" customWidth="1"/>
+    <col min="3" max="3" width="25.33203125" customWidth="1"/>
     <col min="4" max="4" width="22" customWidth="1"/>
-    <col min="5" max="5" width="22.7109375" customWidth="1"/>
+    <col min="5" max="5" width="22.6640625" customWidth="1"/>
     <col min="6" max="6" width="29" customWidth="1"/>
-    <col min="7" max="7" width="27.28515625" customWidth="1"/>
-    <col min="8" max="8" width="27.85546875" customWidth="1"/>
+    <col min="7" max="7" width="27.33203125" customWidth="1"/>
+    <col min="8" max="8" width="27.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="11" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="11" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="12" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="11" t="s">
         <v>6</v>
       </c>
@@ -2737,7 +2731,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="13" t="s">
         <v>8</v>
       </c>
@@ -2757,7 +2751,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="13" t="s">
         <v>10</v>
       </c>
@@ -2774,7 +2768,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="13" t="s">
         <v>13</v>
       </c>
@@ -2788,7 +2782,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="13" t="s">
         <v>15</v>
       </c>
@@ -2802,7 +2796,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="13" t="s">
         <v>17</v>
       </c>
@@ -2810,7 +2804,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="14" t="s">
         <v>19</v>
       </c>
@@ -2818,7 +2812,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="13" t="s">
         <v>21</v>
       </c>
@@ -2827,7 +2821,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="13" t="s">
         <v>23</v>
       </c>
@@ -2835,7 +2829,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="13" t="s">
         <v>25</v>
       </c>
@@ -2846,126 +2840,126 @@
         <v>196</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="20" t="s">
+      <c r="B14" s="18" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="B15" s="20" t="s">
+      <c r="B15" s="18" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="B16" s="20" t="s">
+      <c r="B16" s="18" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="B17" s="20" t="s">
+      <c r="B17" s="18" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="B18" s="20" t="s">
+      <c r="B18" s="18" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="B19" s="20" t="s">
+      <c r="B19" s="18" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="B20" s="20" t="s">
+      <c r="B20" s="18" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="B21" s="20" t="s">
+      <c r="B21" s="18" t="s">
         <v>201</v>
       </c>
       <c r="E21" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="B22" s="20" t="s">
+      <c r="B22" s="18" t="s">
         <v>201</v>
       </c>
       <c r="E22" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="B23" s="20" t="s">
+      <c r="B23" s="18" t="s">
         <v>201</v>
       </c>
       <c r="E23" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="11" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="11" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="11" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" s="11" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="11" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" s="11" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="13" t="s">
         <v>59</v>
       </c>
@@ -2976,7 +2970,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" s="13" t="s">
         <v>61</v>
       </c>
@@ -2984,7 +2978,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="13" t="s">
         <v>63</v>
       </c>
@@ -2992,7 +2986,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" s="15" t="s">
         <v>65</v>
       </c>
@@ -3000,12 +2994,12 @@
         <v>203</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" s="11" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" s="13" t="s">
         <v>70</v>
       </c>
@@ -3016,7 +3010,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" s="13" t="s">
         <v>72</v>
       </c>
@@ -3027,37 +3021,37 @@
         <v>211</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" s="11" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" s="11" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" s="11" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" s="11" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" s="11" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" s="11" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" s="14" t="s">
         <v>86</v>
       </c>
@@ -3065,37 +3059,37 @@
         <v>203</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" s="11" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" s="11" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" s="11" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47" s="11" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48" s="11" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" s="11" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" s="14" t="s">
         <v>99</v>
       </c>
@@ -3103,7 +3097,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" s="14" t="s">
         <v>101</v>
       </c>
@@ -3111,47 +3105,47 @@
         <v>187</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52" s="11" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A53" s="11" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54" s="11" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55" s="11" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A56" s="11" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A57" s="11" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A58" s="11" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A59" s="16" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A60" s="17" t="s">
         <v>119</v>
       </c>
@@ -3162,7 +3156,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A61" s="13" t="s">
         <v>121</v>
       </c>

</xml_diff>